<commit_message>
feat: export MCCC M2E
</commit_message>
<xml_diff>
--- a/public/modeles/Annexe_MCCC_M2E.xlsx
+++ b/public/modeles/Annexe_MCCC_M2E.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davidannebicque/Sites/oreof/public/modeles/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/davidannebicque/Sites/oreof/oreofv1/public/modeles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A3BB730-28BD-514C-B884-E8EDD2745A0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C13D23A-DFDD-C445-9AE3-AF66610EF89F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="modele" sheetId="6" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="175">
   <si>
     <t>ACCREDITATION 2024-2028</t>
   </si>
@@ -177,12 +177,6 @@
   </si>
   <si>
     <t>BC1</t>
-  </si>
-  <si>
-    <t>BC2</t>
-  </si>
-  <si>
-    <t>BC3</t>
   </si>
   <si>
     <t>BC4</t>
@@ -854,7 +848,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="65">
+  <borders count="61">
     <border>
       <left/>
       <right/>
@@ -948,19 +942,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="medium">
@@ -1423,41 +1404,6 @@
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -1673,7 +1619,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="176">
+  <cellXfs count="168">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1778,10 +1724,10 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1795,7 +1741,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1807,7 +1753,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1822,10 +1768,10 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1834,46 +1780,43 @@
     <xf numFmtId="0" fontId="15" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="3" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="5" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1882,10 +1825,7 @@
     <xf numFmtId="0" fontId="23" fillId="5" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -1900,267 +1840,137 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="5" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="5" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="5" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="52" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="52" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="5" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="56" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="60" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="63" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2174,15 +1984,131 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2644,7 +2570,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23720D97-AAF4-46C5-A68F-3C030FC9025A}">
-  <dimension ref="A1:AF28"/>
+  <dimension ref="A1:AC28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.6640625" style="5" customWidth="1"/>
@@ -2661,90 +2587,87 @@
     <col min="19" max="19" width="6.6640625" customWidth="1"/>
     <col min="20" max="20" width="8.33203125" customWidth="1"/>
     <col min="21" max="27" width="14.33203125" customWidth="1"/>
-    <col min="28" max="31" width="5.6640625" customWidth="1"/>
+    <col min="28" max="28" width="5.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="20" x14ac:dyDescent="0.2">
-      <c r="A1" s="168" t="s">
+    <row r="1" spans="1:29" ht="20" x14ac:dyDescent="0.2">
+      <c r="A1" s="122" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="168"/>
-      <c r="C1" s="168"/>
-      <c r="D1" s="168"/>
-      <c r="E1" s="168"/>
-      <c r="F1" s="168"/>
-      <c r="G1" s="168"/>
-      <c r="H1" s="168"/>
-      <c r="I1" s="168"/>
-      <c r="J1" s="168"/>
-      <c r="K1" s="168"/>
-      <c r="L1" s="168"/>
-      <c r="M1" s="168"/>
-      <c r="N1" s="168"/>
-      <c r="O1" s="168"/>
-      <c r="P1" s="168"/>
-      <c r="Q1" s="168"/>
-      <c r="R1" s="168"/>
-      <c r="S1" s="168"/>
-      <c r="T1" s="168"/>
-      <c r="U1" s="168"/>
-      <c r="V1" s="168"/>
-      <c r="W1" s="168"/>
-      <c r="X1" s="168"/>
-      <c r="Y1" s="168"/>
-      <c r="Z1" s="168"/>
-      <c r="AA1" s="168"/>
+      <c r="B1" s="122"/>
+      <c r="C1" s="122"/>
+      <c r="D1" s="122"/>
+      <c r="E1" s="122"/>
+      <c r="F1" s="122"/>
+      <c r="G1" s="122"/>
+      <c r="H1" s="122"/>
+      <c r="I1" s="122"/>
+      <c r="J1" s="122"/>
+      <c r="K1" s="122"/>
+      <c r="L1" s="122"/>
+      <c r="M1" s="122"/>
+      <c r="N1" s="122"/>
+      <c r="O1" s="122"/>
+      <c r="P1" s="122"/>
+      <c r="Q1" s="122"/>
+      <c r="R1" s="122"/>
+      <c r="S1" s="122"/>
+      <c r="T1" s="122"/>
+      <c r="U1" s="122"/>
+      <c r="V1" s="122"/>
+      <c r="W1" s="122"/>
+      <c r="X1" s="122"/>
+      <c r="Y1" s="122"/>
+      <c r="Z1" s="122"/>
+      <c r="AA1" s="122"/>
       <c r="AB1" s="2"/>
-      <c r="AC1" s="2"/>
-      <c r="AD1" s="2"/>
-      <c r="AE1" s="2"/>
-      <c r="AF1" s="30"/>
-    </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.2"/>
-    <row r="3" spans="1:32" ht="18" x14ac:dyDescent="0.2">
-      <c r="A3" s="169" t="s">
+      <c r="AC1" s="30"/>
+    </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.2"/>
+    <row r="3" spans="1:29" ht="18" x14ac:dyDescent="0.2">
+      <c r="A3" s="123" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="169"/>
-      <c r="C3" s="169"/>
-      <c r="D3" s="169"/>
-      <c r="E3" s="169"/>
-      <c r="F3" s="169"/>
-      <c r="G3" s="169"/>
-      <c r="H3" s="169"/>
-      <c r="I3" s="169"/>
-      <c r="J3" s="169"/>
-      <c r="K3" s="169"/>
-      <c r="L3" s="169"/>
-      <c r="M3" s="169"/>
-      <c r="N3" s="169"/>
-      <c r="O3" s="169"/>
-      <c r="P3" s="169"/>
-      <c r="Q3" s="169"/>
-      <c r="R3" s="169"/>
-      <c r="S3" s="169"/>
-      <c r="T3" s="169"/>
-      <c r="U3" s="169"/>
-      <c r="V3" s="169"/>
-      <c r="W3" s="169"/>
-      <c r="X3" s="169"/>
-      <c r="Y3" s="169"/>
-      <c r="Z3" s="169"/>
-      <c r="AA3" s="169"/>
-    </row>
-    <row r="4" spans="1:32" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="5" spans="1:32" ht="16" x14ac:dyDescent="0.2">
+      <c r="B3" s="123"/>
+      <c r="C3" s="123"/>
+      <c r="D3" s="123"/>
+      <c r="E3" s="123"/>
+      <c r="F3" s="123"/>
+      <c r="G3" s="123"/>
+      <c r="H3" s="123"/>
+      <c r="I3" s="123"/>
+      <c r="J3" s="123"/>
+      <c r="K3" s="123"/>
+      <c r="L3" s="123"/>
+      <c r="M3" s="123"/>
+      <c r="N3" s="123"/>
+      <c r="O3" s="123"/>
+      <c r="P3" s="123"/>
+      <c r="Q3" s="123"/>
+      <c r="R3" s="123"/>
+      <c r="S3" s="123"/>
+      <c r="T3" s="123"/>
+      <c r="U3" s="123"/>
+      <c r="V3" s="123"/>
+      <c r="W3" s="123"/>
+      <c r="X3" s="123"/>
+      <c r="Y3" s="123"/>
+      <c r="Z3" s="123"/>
+      <c r="AA3" s="123"/>
+    </row>
+    <row r="4" spans="1:29" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="5" spans="1:29" ht="16" x14ac:dyDescent="0.2">
       <c r="F5" s="32"/>
-      <c r="G5" s="170" t="s">
+      <c r="G5" s="124" t="s">
         <v>2</v>
       </c>
-      <c r="H5" s="170"/>
-      <c r="I5" s="170"/>
-      <c r="J5" s="171" t="s">
-        <v>176</v>
-      </c>
-      <c r="K5" s="171"/>
-      <c r="L5" s="171"/>
+      <c r="H5" s="124"/>
+      <c r="I5" s="124"/>
+      <c r="J5" s="125" t="s">
+        <v>174</v>
+      </c>
+      <c r="K5" s="125"/>
+      <c r="L5" s="125"/>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
@@ -2753,40 +2676,40 @@
       <c r="S5" s="2"/>
       <c r="T5" s="2"/>
     </row>
-    <row r="6" spans="1:32" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:29" ht="16" x14ac:dyDescent="0.2">
       <c r="B6" s="33"/>
       <c r="C6" s="34"/>
       <c r="D6" s="34"/>
       <c r="E6" s="34"/>
       <c r="F6" s="32"/>
-      <c r="G6" s="170" t="s">
+      <c r="G6" s="124" t="s">
         <v>3</v>
       </c>
-      <c r="H6" s="170"/>
-      <c r="I6" s="170"/>
-      <c r="J6" s="171" t="s">
-        <v>175</v>
-      </c>
-      <c r="K6" s="171"/>
-      <c r="L6" s="171"/>
-      <c r="M6" s="171"/>
-      <c r="N6" s="171"/>
-      <c r="O6" s="171"/>
-      <c r="P6" s="171"/>
-      <c r="Q6" s="171"/>
-      <c r="R6" s="171"/>
-      <c r="S6" s="171"/>
-      <c r="T6" s="171"/>
-      <c r="U6" s="171"/>
-      <c r="V6" s="171"/>
+      <c r="H6" s="124"/>
+      <c r="I6" s="124"/>
+      <c r="J6" s="125" t="s">
+        <v>173</v>
+      </c>
+      <c r="K6" s="125"/>
+      <c r="L6" s="125"/>
+      <c r="M6" s="125"/>
+      <c r="N6" s="125"/>
+      <c r="O6" s="125"/>
+      <c r="P6" s="125"/>
+      <c r="Q6" s="125"/>
+      <c r="R6" s="125"/>
+      <c r="S6" s="125"/>
+      <c r="T6" s="125"/>
+      <c r="U6" s="125"/>
+      <c r="V6" s="125"/>
       <c r="W6" s="34"/>
     </row>
-    <row r="7" spans="1:32" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:29" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="35"/>
       <c r="B7" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="73" t="s">
+      <c r="C7" s="71" t="s">
         <v>5</v>
       </c>
       <c r="D7" s="37" t="s">
@@ -2794,30 +2717,29 @@
       </c>
       <c r="E7" s="35"/>
       <c r="F7" s="32"/>
-      <c r="G7" s="170" t="s">
+      <c r="G7" s="124" t="s">
         <v>7</v>
       </c>
-      <c r="H7" s="170"/>
-      <c r="I7" s="170"/>
-      <c r="J7" s="171" t="s">
-        <v>174</v>
-      </c>
-      <c r="K7" s="171"/>
-      <c r="L7" s="171"/>
-      <c r="M7" s="171"/>
-      <c r="N7" s="171"/>
-      <c r="O7" s="171"/>
-      <c r="P7" s="171"/>
-      <c r="Q7" s="171"/>
-      <c r="R7" s="171"/>
-      <c r="S7" s="171"/>
-      <c r="T7" s="171"/>
-      <c r="U7" s="171"/>
-      <c r="V7" s="171"/>
+      <c r="H7" s="124"/>
+      <c r="I7" s="124"/>
+      <c r="J7" s="125" t="s">
+        <v>172</v>
+      </c>
+      <c r="K7" s="125"/>
+      <c r="L7" s="125"/>
+      <c r="M7" s="125"/>
+      <c r="N7" s="125"/>
+      <c r="O7" s="125"/>
+      <c r="P7" s="125"/>
+      <c r="Q7" s="125"/>
+      <c r="R7" s="125"/>
+      <c r="S7" s="125"/>
+      <c r="T7" s="125"/>
+      <c r="U7" s="125"/>
+      <c r="V7" s="125"/>
       <c r="AB7" s="3"/>
-      <c r="AC7" s="3"/>
-    </row>
-    <row r="8" spans="1:32" ht="8.5" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:29" ht="8.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C8" s="35"/>
       <c r="D8" s="31"/>
       <c r="E8" s="31"/>
@@ -2841,10 +2763,9 @@
       <c r="W8" s="34"/>
       <c r="Z8" s="34"/>
       <c r="AB8" s="3"/>
-      <c r="AC8" s="3"/>
-    </row>
-    <row r="9" spans="1:32" ht="16" x14ac:dyDescent="0.2">
-      <c r="C9" s="73" t="s">
+    </row>
+    <row r="9" spans="1:29" ht="16" x14ac:dyDescent="0.2">
+      <c r="C9" s="71" t="s">
         <v>5</v>
       </c>
       <c r="D9" s="37" t="s">
@@ -2852,16 +2773,16 @@
       </c>
       <c r="E9" s="35"/>
       <c r="F9" s="32"/>
-      <c r="G9" s="170" t="s">
+      <c r="G9" s="124" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="170"/>
-      <c r="I9" s="170"/>
-      <c r="J9" s="171" t="s">
-        <v>173</v>
-      </c>
-      <c r="K9" s="171"/>
-      <c r="L9" s="171"/>
+      <c r="H9" s="124"/>
+      <c r="I9" s="124"/>
+      <c r="J9" s="125" t="s">
+        <v>171</v>
+      </c>
+      <c r="K9" s="125"/>
+      <c r="L9" s="125"/>
       <c r="M9" s="3"/>
       <c r="N9" s="3"/>
       <c r="O9" s="3"/>
@@ -2874,11 +2795,8 @@
       <c r="V9" s="4"/>
       <c r="W9" s="38"/>
       <c r="AB9" s="3"/>
-      <c r="AC9" s="3"/>
-      <c r="AD9" s="3"/>
-      <c r="AE9" s="3"/>
-    </row>
-    <row r="10" spans="1:32" ht="5" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="1:29" ht="5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C10" s="39"/>
       <c r="D10" s="40"/>
       <c r="E10" s="40"/>
@@ -2891,26 +2809,26 @@
       <c r="L10" s="19"/>
       <c r="M10" s="22"/>
     </row>
-    <row r="11" spans="1:32" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:29" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C11" s="36"/>
       <c r="D11" s="37" t="s">
         <v>11</v>
       </c>
       <c r="E11" s="35"/>
       <c r="F11" s="32"/>
-      <c r="G11" s="170" t="s">
+      <c r="G11" s="124" t="s">
         <v>12</v>
       </c>
-      <c r="H11" s="170"/>
-      <c r="I11" s="170"/>
-      <c r="J11" s="171" t="s">
-        <v>172</v>
-      </c>
-      <c r="K11" s="171"/>
-      <c r="L11" s="171"/>
+      <c r="H11" s="124"/>
+      <c r="I11" s="124"/>
+      <c r="J11" s="125" t="s">
+        <v>170</v>
+      </c>
+      <c r="K11" s="125"/>
+      <c r="L11" s="125"/>
       <c r="M11" s="23"/>
     </row>
-    <row r="12" spans="1:32" ht="5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:29" ht="5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C12" s="31"/>
       <c r="D12" s="31"/>
       <c r="E12" s="31"/>
@@ -2923,26 +2841,26 @@
       <c r="L12" s="19"/>
       <c r="M12" s="23"/>
     </row>
-    <row r="13" spans="1:32" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:29" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C13" s="36"/>
       <c r="D13" s="37" t="s">
         <v>14</v>
       </c>
       <c r="E13" s="35"/>
       <c r="F13" s="32"/>
-      <c r="G13" s="170" t="s">
+      <c r="G13" s="124" t="s">
         <v>15</v>
       </c>
-      <c r="H13" s="170"/>
-      <c r="I13" s="170"/>
-      <c r="J13" s="171" t="s">
-        <v>171</v>
-      </c>
-      <c r="K13" s="171"/>
-      <c r="L13" s="171"/>
+      <c r="H13" s="124"/>
+      <c r="I13" s="124"/>
+      <c r="J13" s="125" t="s">
+        <v>169</v>
+      </c>
+      <c r="K13" s="125"/>
+      <c r="L13" s="125"/>
       <c r="M13" s="23"/>
     </row>
-    <row r="14" spans="1:32" ht="11" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:29" ht="11" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C14" s="5"/>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
@@ -2970,109 +2888,100 @@
       <c r="AA14" s="5"/>
       <c r="AB14" s="5"/>
       <c r="AC14" s="5"/>
-      <c r="AD14" s="5"/>
-      <c r="AE14" s="5"/>
-      <c r="AF14" s="5"/>
-    </row>
-    <row r="15" spans="1:32" s="41" customFormat="1" ht="11" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="161" t="s">
+    </row>
+    <row r="15" spans="1:29" s="41" customFormat="1" ht="11" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="130" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="162"/>
-      <c r="C15" s="165" t="s">
+      <c r="B15" s="131"/>
+      <c r="C15" s="134" t="s">
         <v>17</v>
       </c>
-      <c r="D15" s="165"/>
-      <c r="E15" s="165"/>
-      <c r="F15" s="165"/>
-      <c r="G15" s="165"/>
-      <c r="H15" s="165"/>
-      <c r="I15" s="165"/>
-      <c r="J15" s="162"/>
-      <c r="K15" s="146" t="s">
+      <c r="D15" s="134"/>
+      <c r="E15" s="134"/>
+      <c r="F15" s="134"/>
+      <c r="G15" s="134"/>
+      <c r="H15" s="134"/>
+      <c r="I15" s="134"/>
+      <c r="J15" s="131"/>
+      <c r="K15" s="136" t="s">
         <v>18</v>
       </c>
-      <c r="L15" s="147"/>
-      <c r="M15" s="147"/>
-      <c r="N15" s="147"/>
-      <c r="O15" s="147"/>
-      <c r="P15" s="147"/>
-      <c r="Q15" s="147"/>
-      <c r="R15" s="147"/>
-      <c r="S15" s="147"/>
-      <c r="T15" s="167"/>
-      <c r="U15" s="147" t="s">
+      <c r="L15" s="137"/>
+      <c r="M15" s="137"/>
+      <c r="N15" s="137"/>
+      <c r="O15" s="137"/>
+      <c r="P15" s="137"/>
+      <c r="Q15" s="137"/>
+      <c r="R15" s="137"/>
+      <c r="S15" s="137"/>
+      <c r="T15" s="138"/>
+      <c r="U15" s="137" t="s">
         <v>19</v>
       </c>
-      <c r="V15" s="147"/>
-      <c r="W15" s="167"/>
-      <c r="X15" s="145" t="s">
+      <c r="V15" s="137"/>
+      <c r="W15" s="138"/>
+      <c r="X15" s="158" t="s">
         <v>20</v>
       </c>
-      <c r="Y15" s="145"/>
-      <c r="Z15" s="145"/>
-      <c r="AA15" s="145"/>
-      <c r="AB15" s="122" t="s">
+      <c r="Y15" s="158"/>
+      <c r="Z15" s="158"/>
+      <c r="AA15" s="158"/>
+      <c r="AB15" s="139" t="s">
         <v>31</v>
       </c>
-      <c r="AC15" s="123"/>
-      <c r="AD15" s="123"/>
-      <c r="AE15" s="124"/>
-    </row>
-    <row r="16" spans="1:32" s="41" customFormat="1" ht="11" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="163"/>
-      <c r="B16" s="164"/>
-      <c r="C16" s="166"/>
-      <c r="D16" s="166"/>
-      <c r="E16" s="166"/>
-      <c r="F16" s="166"/>
-      <c r="G16" s="166"/>
-      <c r="H16" s="166"/>
-      <c r="I16" s="166"/>
-      <c r="J16" s="164"/>
-      <c r="K16" s="146" t="s">
+    </row>
+    <row r="16" spans="1:29" s="41" customFormat="1" ht="11" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="132"/>
+      <c r="B16" s="133"/>
+      <c r="C16" s="135"/>
+      <c r="D16" s="135"/>
+      <c r="E16" s="135"/>
+      <c r="F16" s="135"/>
+      <c r="G16" s="135"/>
+      <c r="H16" s="135"/>
+      <c r="I16" s="135"/>
+      <c r="J16" s="133"/>
+      <c r="K16" s="136" t="s">
         <v>21</v>
       </c>
-      <c r="L16" s="147"/>
-      <c r="M16" s="147"/>
-      <c r="N16" s="148"/>
-      <c r="O16" s="146" t="s">
+      <c r="L16" s="137"/>
+      <c r="M16" s="137"/>
+      <c r="N16" s="159"/>
+      <c r="O16" s="136" t="s">
         <v>22</v>
       </c>
-      <c r="P16" s="147"/>
-      <c r="Q16" s="147"/>
-      <c r="R16" s="148"/>
-      <c r="S16" s="149" t="s">
+      <c r="P16" s="137"/>
+      <c r="Q16" s="137"/>
+      <c r="R16" s="159"/>
+      <c r="S16" s="160" t="s">
         <v>23</v>
       </c>
-      <c r="T16" s="151" t="s">
+      <c r="T16" s="162" t="s">
         <v>24</v>
       </c>
-      <c r="U16" s="153" t="s">
+      <c r="U16" s="164" t="s">
         <v>25</v>
       </c>
-      <c r="V16" s="155" t="s">
+      <c r="V16" s="128" t="s">
         <v>26</v>
       </c>
-      <c r="W16" s="157" t="s">
+      <c r="W16" s="166" t="s">
         <v>27</v>
       </c>
-      <c r="X16" s="159" t="s">
+      <c r="X16" s="126" t="s">
         <v>28</v>
       </c>
-      <c r="Y16" s="160"/>
-      <c r="Z16" s="155" t="s">
+      <c r="Y16" s="127"/>
+      <c r="Z16" s="128" t="s">
         <v>29</v>
       </c>
-      <c r="AA16" s="143" t="s">
+      <c r="AA16" s="156" t="s">
         <v>30</v>
       </c>
-      <c r="AB16" s="125"/>
-      <c r="AC16" s="126"/>
-      <c r="AD16" s="126"/>
-      <c r="AE16" s="127"/>
-    </row>
-    <row r="17" spans="1:31" s="42" customFormat="1" ht="68" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="AB16" s="140"/>
+    </row>
+    <row r="17" spans="1:28" s="42" customFormat="1" ht="68" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A17" s="52" t="s">
         <v>32</v>
       </c>
@@ -3086,19 +2995,19 @@
         <v>35</v>
       </c>
       <c r="E17" s="53" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="F17" s="53" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="G17" s="47" t="s">
         <v>36</v>
       </c>
       <c r="H17" s="47" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="I17" s="47" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J17" s="65" t="s">
         <v>37</v>
@@ -3127,259 +3036,227 @@
       <c r="R17" s="55" t="s">
         <v>42</v>
       </c>
-      <c r="S17" s="150"/>
-      <c r="T17" s="152"/>
-      <c r="U17" s="154"/>
-      <c r="V17" s="156"/>
-      <c r="W17" s="158"/>
+      <c r="S17" s="161"/>
+      <c r="T17" s="163"/>
+      <c r="U17" s="165"/>
+      <c r="V17" s="129"/>
+      <c r="W17" s="167"/>
       <c r="X17" s="66" t="s">
         <v>43</v>
       </c>
       <c r="Y17" s="58" t="s">
         <v>44</v>
       </c>
-      <c r="Z17" s="156"/>
-      <c r="AA17" s="144"/>
-      <c r="AB17" s="114" t="s">
+      <c r="Z17" s="129"/>
+      <c r="AA17" s="157"/>
+      <c r="AB17" s="110" t="s">
         <v>45</v>
       </c>
-      <c r="AC17" s="68" t="s">
-        <v>46</v>
-      </c>
-      <c r="AD17" s="68" t="s">
+    </row>
+    <row r="18" spans="1:28" ht="29" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="98" t="s">
         <v>47</v>
       </c>
-      <c r="AE17" s="69" t="s">
+      <c r="B18" s="99" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="18" spans="1:31" ht="29" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="102" t="s">
+      <c r="C18" s="98" t="s">
         <v>49</v>
       </c>
-      <c r="B18" s="103" t="s">
+      <c r="D18" s="99" t="s">
         <v>50</v>
       </c>
-      <c r="C18" s="102" t="s">
+      <c r="E18" s="78"/>
+      <c r="F18" s="78"/>
+      <c r="G18" s="79" t="s">
         <v>51</v>
       </c>
-      <c r="D18" s="103" t="s">
-        <v>52</v>
-      </c>
-      <c r="E18" s="80"/>
-      <c r="F18" s="80"/>
-      <c r="G18" s="81" t="s">
-        <v>53</v>
-      </c>
-      <c r="H18" s="120"/>
-      <c r="I18" s="120"/>
-      <c r="J18" s="78">
+      <c r="H18" s="116"/>
+      <c r="I18" s="116"/>
+      <c r="J18" s="76">
         <v>37</v>
       </c>
-      <c r="K18" s="82"/>
-      <c r="L18" s="83">
+      <c r="K18" s="80"/>
+      <c r="L18" s="81">
         <v>61</v>
       </c>
-      <c r="M18" s="84"/>
-      <c r="N18" s="77">
+      <c r="M18" s="82"/>
+      <c r="N18" s="75">
         <v>61</v>
       </c>
-      <c r="O18" s="82"/>
-      <c r="P18" s="83"/>
-      <c r="Q18" s="84"/>
-      <c r="R18" s="77"/>
-      <c r="S18" s="77"/>
-      <c r="T18" s="79">
+      <c r="O18" s="80"/>
+      <c r="P18" s="81"/>
+      <c r="Q18" s="82"/>
+      <c r="R18" s="75"/>
+      <c r="S18" s="75"/>
+      <c r="T18" s="77">
         <v>216</v>
       </c>
-      <c r="U18" s="111" t="s">
+      <c r="U18" s="107" t="s">
         <v>5</v>
       </c>
-      <c r="V18" s="104"/>
-      <c r="W18" s="112"/>
-      <c r="X18" s="113"/>
-      <c r="Y18" s="105"/>
-      <c r="Z18" s="106"/>
-      <c r="AA18" s="115"/>
-      <c r="AB18" s="116">
+      <c r="V18" s="100"/>
+      <c r="W18" s="108"/>
+      <c r="X18" s="109"/>
+      <c r="Y18" s="101"/>
+      <c r="Z18" s="102"/>
+      <c r="AA18" s="111"/>
+      <c r="AB18" s="112">
         <v>1</v>
       </c>
-      <c r="AC18" s="100"/>
-      <c r="AD18" s="100"/>
-      <c r="AE18" s="101"/>
-    </row>
-    <row r="19" spans="1:31" ht="44" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="90"/>
-      <c r="B19" s="91"/>
-      <c r="C19" s="91"/>
-      <c r="D19" s="92" t="s">
-        <v>57</v>
-      </c>
-      <c r="E19" s="93"/>
-      <c r="F19" s="93"/>
-      <c r="G19" s="94"/>
-      <c r="H19" s="121"/>
-      <c r="I19" s="121"/>
-      <c r="J19" s="95">
+    </row>
+    <row r="19" spans="1:28" ht="44" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="88"/>
+      <c r="B19" s="89"/>
+      <c r="C19" s="89"/>
+      <c r="D19" s="90" t="s">
+        <v>55</v>
+      </c>
+      <c r="E19" s="91"/>
+      <c r="F19" s="91"/>
+      <c r="G19" s="92"/>
+      <c r="H19" s="117"/>
+      <c r="I19" s="117"/>
+      <c r="J19" s="93">
         <f>SUM(J18:J18)</f>
         <v>37</v>
       </c>
-      <c r="K19" s="70"/>
-      <c r="L19" s="71">
+      <c r="K19" s="68"/>
+      <c r="L19" s="69">
         <f>SUM(L18:L18)</f>
         <v>61</v>
       </c>
-      <c r="M19" s="72">
+      <c r="M19" s="70">
         <f>SUM(M18:M18)</f>
         <v>0</v>
       </c>
-      <c r="N19" s="96">
+      <c r="N19" s="94">
         <f>SUM(N18:N18)</f>
         <v>61</v>
       </c>
-      <c r="O19" s="97"/>
-      <c r="P19" s="71"/>
-      <c r="Q19" s="98"/>
-      <c r="R19" s="99"/>
-      <c r="S19" s="99"/>
-      <c r="T19" s="95">
+      <c r="O19" s="95"/>
+      <c r="P19" s="69"/>
+      <c r="Q19" s="96"/>
+      <c r="R19" s="97"/>
+      <c r="S19" s="97"/>
+      <c r="T19" s="93">
         <v>216</v>
       </c>
-      <c r="U19" s="134"/>
-      <c r="V19" s="135"/>
-      <c r="W19" s="135"/>
-      <c r="X19" s="136"/>
-      <c r="Y19" s="137"/>
-      <c r="Z19" s="138"/>
-      <c r="AA19" s="139"/>
-      <c r="AB19" s="117"/>
-    </row>
-    <row r="20" spans="1:31" ht="44" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="85"/>
-      <c r="B20" s="85"/>
+      <c r="U19" s="147"/>
+      <c r="V19" s="148"/>
+      <c r="W19" s="148"/>
+      <c r="X19" s="149"/>
+      <c r="Y19" s="150"/>
+      <c r="Z19" s="151"/>
+      <c r="AA19" s="152"/>
+      <c r="AB19" s="113"/>
+    </row>
+    <row r="20" spans="1:28" ht="44" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="83"/>
+      <c r="B20" s="83"/>
       <c r="C20" s="1"/>
       <c r="D20" s="50"/>
       <c r="E20" s="50"/>
       <c r="F20" s="50"/>
-      <c r="J20" s="86"/>
+      <c r="J20" s="84"/>
       <c r="K20" s="59"/>
       <c r="L20" s="60"/>
       <c r="M20" s="61"/>
-      <c r="N20" s="87"/>
+      <c r="N20" s="85"/>
       <c r="O20" s="59"/>
       <c r="P20" s="60"/>
       <c r="Q20" s="61"/>
-      <c r="R20" s="87"/>
-      <c r="S20" s="88"/>
-      <c r="T20" s="89"/>
-      <c r="U20" s="107"/>
-      <c r="V20" s="108"/>
-      <c r="W20" s="110"/>
-      <c r="X20" s="107"/>
-      <c r="Y20" s="108"/>
-      <c r="Z20" s="109"/>
-      <c r="AA20" s="118"/>
-      <c r="AB20" s="119"/>
-    </row>
-    <row r="21" spans="1:31" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="R20" s="85"/>
+      <c r="S20" s="86"/>
+      <c r="T20" s="87"/>
+      <c r="U20" s="103"/>
+      <c r="V20" s="104"/>
+      <c r="W20" s="106"/>
+      <c r="X20" s="103"/>
+      <c r="Y20" s="104"/>
+      <c r="Z20" s="105"/>
+      <c r="AA20" s="114"/>
+      <c r="AB20" s="115"/>
+    </row>
+    <row r="21" spans="1:28" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="48"/>
       <c r="B21" s="48"/>
       <c r="J21" s="56"/>
-      <c r="K21" s="140"/>
-      <c r="L21" s="141"/>
-      <c r="M21" s="141"/>
-      <c r="N21" s="141"/>
-      <c r="O21" s="141"/>
-      <c r="P21" s="141"/>
-      <c r="Q21" s="141"/>
-      <c r="R21" s="141"/>
-      <c r="S21" s="142"/>
+      <c r="K21" s="153"/>
+      <c r="L21" s="154"/>
+      <c r="M21" s="154"/>
+      <c r="N21" s="154"/>
+      <c r="O21" s="154"/>
+      <c r="P21" s="154"/>
+      <c r="Q21" s="154"/>
+      <c r="R21" s="154"/>
+      <c r="S21" s="155"/>
       <c r="T21" s="43"/>
     </row>
-    <row r="22" spans="1:31" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:28" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="49"/>
       <c r="B22" s="49"/>
       <c r="C22" s="50"/>
       <c r="J22" s="56"/>
-      <c r="K22" s="131"/>
-      <c r="L22" s="132"/>
-      <c r="M22" s="132"/>
-      <c r="N22" s="132"/>
-      <c r="O22" s="132"/>
-      <c r="P22" s="132"/>
-      <c r="Q22" s="132"/>
-      <c r="R22" s="132"/>
-      <c r="S22" s="132"/>
-      <c r="T22" s="133"/>
-    </row>
-    <row r="23" spans="1:31" ht="31.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="K22" s="144"/>
+      <c r="L22" s="145"/>
+      <c r="M22" s="145"/>
+      <c r="N22" s="145"/>
+      <c r="O22" s="145"/>
+      <c r="P22" s="145"/>
+      <c r="Q22" s="145"/>
+      <c r="R22" s="145"/>
+      <c r="S22" s="145"/>
+      <c r="T22" s="146"/>
+    </row>
+    <row r="23" spans="1:28" ht="31.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="J23" s="56"/>
-      <c r="K23" s="131"/>
-      <c r="L23" s="132"/>
-      <c r="M23" s="132"/>
-      <c r="N23" s="132"/>
-      <c r="O23" s="132"/>
-      <c r="P23" s="132"/>
-      <c r="Q23" s="132"/>
-      <c r="R23" s="132"/>
-      <c r="S23" s="133"/>
+      <c r="K23" s="144"/>
+      <c r="L23" s="145"/>
+      <c r="M23" s="145"/>
+      <c r="N23" s="145"/>
+      <c r="O23" s="145"/>
+      <c r="P23" s="145"/>
+      <c r="Q23" s="145"/>
+      <c r="R23" s="145"/>
+      <c r="S23" s="146"/>
       <c r="T23" s="43"/>
     </row>
-    <row r="24" spans="1:31" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="1:31" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:28" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B25" s="44"/>
       <c r="D25" s="44" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="W25" s="10"/>
       <c r="X25" s="45" t="s">
-        <v>59</v>
-      </c>
-      <c r="Y25" s="128"/>
-      <c r="Z25" s="129"/>
-      <c r="AA25" s="130"/>
-    </row>
-    <row r="26" spans="1:31" ht="34.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+        <v>57</v>
+      </c>
+      <c r="Y25" s="141"/>
+      <c r="Z25" s="142"/>
+      <c r="AA25" s="143"/>
+    </row>
+    <row r="26" spans="1:28" ht="34.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A26" s="10"/>
       <c r="B26" s="45"/>
       <c r="D26" s="45" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="W26" s="46"/>
       <c r="X26" s="45" t="s">
-        <v>61</v>
-      </c>
-      <c r="Y26" s="128"/>
-      <c r="Z26" s="129"/>
-      <c r="AA26" s="130"/>
-    </row>
-    <row r="28" spans="1:31" ht="111" customHeight="1" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+      <c r="Y26" s="141"/>
+      <c r="Z26" s="142"/>
+      <c r="AA26" s="143"/>
+    </row>
+    <row r="28" spans="1:28" ht="111" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="50"/>
       <c r="B28" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="A1:AA1"/>
-    <mergeCell ref="A3:AA3"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="J13:L13"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J6:V6"/>
-    <mergeCell ref="J7:V7"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="J9:L9"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="J5:L5"/>
-    <mergeCell ref="X16:Y16"/>
-    <mergeCell ref="Z16:Z17"/>
-    <mergeCell ref="A15:B16"/>
-    <mergeCell ref="C15:J16"/>
-    <mergeCell ref="K15:T15"/>
-    <mergeCell ref="U15:W15"/>
-    <mergeCell ref="AB15:AE16"/>
+    <mergeCell ref="AB15:AB16"/>
     <mergeCell ref="Y26:AA26"/>
     <mergeCell ref="K22:T22"/>
     <mergeCell ref="K23:S23"/>
@@ -3395,6 +3272,26 @@
     <mergeCell ref="U16:U17"/>
     <mergeCell ref="V16:V17"/>
     <mergeCell ref="W16:W17"/>
+    <mergeCell ref="X16:Y16"/>
+    <mergeCell ref="Z16:Z17"/>
+    <mergeCell ref="A15:B16"/>
+    <mergeCell ref="C15:J16"/>
+    <mergeCell ref="K15:T15"/>
+    <mergeCell ref="U15:W15"/>
+    <mergeCell ref="A1:AA1"/>
+    <mergeCell ref="A3:AA3"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="J13:L13"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J6:V6"/>
+    <mergeCell ref="J7:V7"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="J9:L9"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="J5:L5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3412,13 +3309,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:51" ht="20" x14ac:dyDescent="0.2">
-      <c r="A1" s="174" t="s">
+      <c r="A1" s="120" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="174"/>
-      <c r="C1" s="174"/>
-      <c r="D1" s="174"/>
-      <c r="E1" s="174"/>
+      <c r="B1" s="120"/>
+      <c r="C1" s="120"/>
+      <c r="D1" s="120"/>
+      <c r="E1" s="120"/>
       <c r="F1" s="7"/>
       <c r="G1" s="7"/>
       <c r="H1" s="7"/>
@@ -3457,13 +3354,13 @@
       <c r="AY1" s="2"/>
     </row>
     <row r="2" spans="1:51" ht="18" x14ac:dyDescent="0.2">
-      <c r="A2" s="175" t="s">
-        <v>62</v>
-      </c>
-      <c r="B2" s="175"/>
-      <c r="C2" s="175"/>
-      <c r="D2" s="175"/>
-      <c r="E2" s="175"/>
+      <c r="A2" s="121" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="121"/>
+      <c r="C2" s="121"/>
+      <c r="D2" s="121"/>
+      <c r="E2" s="121"/>
       <c r="F2" s="8"/>
       <c r="G2" s="8"/>
       <c r="H2" s="8"/>
@@ -3484,13 +3381,13 @@
       <c r="W2" s="8"/>
     </row>
     <row r="3" spans="1:51" ht="18" x14ac:dyDescent="0.2">
-      <c r="A3" s="175" t="s">
+      <c r="A3" s="121" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="175"/>
-      <c r="C3" s="175"/>
-      <c r="D3" s="175"/>
-      <c r="E3" s="175"/>
+      <c r="B3" s="121"/>
+      <c r="C3" s="121"/>
+      <c r="D3" s="121"/>
+      <c r="E3" s="121"/>
       <c r="F3" s="8"/>
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
@@ -3526,7 +3423,7 @@
         <v>2</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E5" s="9"/>
       <c r="F5" s="13"/>
@@ -3549,7 +3446,7 @@
         <v>3</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E6" s="9"/>
       <c r="F6" s="13"/>
@@ -3731,7 +3628,7 @@
         <v>15</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E13" s="9"/>
       <c r="F13" s="13"/>
@@ -3749,468 +3646,468 @@
     </row>
     <row r="16" spans="1:51" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="26" t="s">
-        <v>66</v>
-      </c>
-      <c r="B16" s="172" t="s">
-        <v>50</v>
-      </c>
-      <c r="C16" s="173"/>
+        <v>64</v>
+      </c>
+      <c r="B16" s="118" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" s="119"/>
       <c r="F16" s="62"/>
     </row>
     <row r="17" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="27"/>
       <c r="B17" s="28" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C17" s="67" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F17" s="62"/>
     </row>
     <row r="18" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="27"/>
       <c r="B18" s="28" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C18" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F18" s="62"/>
     </row>
     <row r="19" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="28" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C19" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F19" s="62"/>
     </row>
     <row r="20" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="28" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C20" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F20" s="62"/>
     </row>
     <row r="21" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="28" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C21" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F21" s="62"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B22" s="28" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C22" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B23" s="28" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C23" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B24" s="28" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C24" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B25" s="28" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C25" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B26" s="28" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C26" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="26" t="s">
-        <v>87</v>
-      </c>
-      <c r="B27" s="172" t="s">
-        <v>54</v>
-      </c>
-      <c r="C27" s="173"/>
+        <v>85</v>
+      </c>
+      <c r="B27" s="118" t="s">
+        <v>52</v>
+      </c>
+      <c r="C27" s="119"/>
     </row>
     <row r="28" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="27"/>
       <c r="B28" s="28" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C28" s="29" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="27"/>
       <c r="B29" s="28" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C29" s="29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="27"/>
       <c r="B30" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="C30" s="29" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B31" s="72" t="s">
         <v>92</v>
       </c>
-      <c r="C30" s="29" t="s">
+      <c r="C31" t="s">
         <v>93</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B31" s="74" t="s">
-        <v>94</v>
-      </c>
-      <c r="C31" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="26"/>
-      <c r="B32" s="75" t="s">
-        <v>96</v>
+      <c r="B32" s="73" t="s">
+        <v>94</v>
       </c>
       <c r="C32" s="27" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="27"/>
-      <c r="B33" s="74" t="s">
-        <v>98</v>
+      <c r="B33" s="72" t="s">
+        <v>96</v>
       </c>
       <c r="C33" s="29" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="27"/>
-      <c r="B34" s="74" t="s">
-        <v>100</v>
+      <c r="B34" s="72" t="s">
+        <v>98</v>
       </c>
       <c r="C34" s="29" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="27"/>
-      <c r="B35" s="74" t="s">
-        <v>102</v>
+      <c r="B35" s="72" t="s">
+        <v>100</v>
       </c>
       <c r="C35" s="29" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="27"/>
-      <c r="B36" s="74" t="s">
-        <v>104</v>
+      <c r="B36" s="72" t="s">
+        <v>102</v>
       </c>
       <c r="C36" s="29" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="27"/>
-      <c r="B37" s="74" t="s">
-        <v>106</v>
+      <c r="B37" s="72" t="s">
+        <v>104</v>
       </c>
       <c r="C37" s="29" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="27"/>
-      <c r="B38" s="74" t="s">
-        <v>108</v>
+      <c r="B38" s="72" t="s">
+        <v>106</v>
       </c>
       <c r="C38" s="29" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A39" s="27"/>
-      <c r="B39" s="74" t="s">
-        <v>110</v>
+      <c r="B39" s="72" t="s">
+        <v>108</v>
       </c>
       <c r="C39" s="29" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="27"/>
-      <c r="B40" s="74" t="s">
-        <v>112</v>
+      <c r="B40" s="72" t="s">
+        <v>110</v>
       </c>
       <c r="C40" s="29" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="27"/>
-      <c r="B41" s="74" t="s">
-        <v>114</v>
+      <c r="B41" s="72" t="s">
+        <v>112</v>
       </c>
       <c r="C41" s="29" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="27"/>
-      <c r="B42" s="74" t="s">
-        <v>116</v>
+      <c r="B42" s="72" t="s">
+        <v>114</v>
       </c>
       <c r="C42" s="29" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="27"/>
-      <c r="B43" s="74" t="s">
-        <v>118</v>
+      <c r="B43" s="72" t="s">
+        <v>116</v>
       </c>
       <c r="C43" s="29" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="27"/>
-      <c r="B44" s="74" t="s">
-        <v>120</v>
+      <c r="B44" s="72" t="s">
+        <v>118</v>
       </c>
       <c r="C44" s="29" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="27"/>
-      <c r="B45" s="74" t="s">
-        <v>122</v>
+      <c r="B45" s="72" t="s">
+        <v>120</v>
       </c>
       <c r="C45" s="29" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" s="26" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B46" s="51" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C46" s="29"/>
     </row>
     <row r="47" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" s="26"/>
-      <c r="B47" s="74" t="s">
-        <v>125</v>
+      <c r="B47" s="72" t="s">
+        <v>123</v>
       </c>
       <c r="C47" s="29" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" s="26"/>
-      <c r="B48" s="74" t="s">
-        <v>127</v>
+      <c r="B48" s="72" t="s">
+        <v>125</v>
       </c>
       <c r="C48" s="29" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" s="26"/>
-      <c r="B49" s="74" t="s">
-        <v>129</v>
+      <c r="B49" s="72" t="s">
+        <v>127</v>
       </c>
       <c r="C49" s="29" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A50" s="26"/>
-      <c r="B50" s="74" t="s">
-        <v>131</v>
+      <c r="B50" s="72" t="s">
+        <v>129</v>
       </c>
       <c r="C50" s="29" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A51" s="26"/>
-      <c r="B51" s="74" t="s">
-        <v>133</v>
+      <c r="B51" s="72" t="s">
+        <v>131</v>
       </c>
       <c r="C51" s="29" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" s="27"/>
-      <c r="B52" s="74" t="s">
+      <c r="B52" s="72" t="s">
+        <v>133</v>
+      </c>
+      <c r="C52" s="29" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B53" s="72" t="s">
         <v>135</v>
       </c>
-      <c r="C52" s="29" t="s">
+      <c r="C53" t="s">
         <v>136</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B53" s="74" t="s">
-        <v>137</v>
-      </c>
-      <c r="C53" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A54" s="26"/>
-      <c r="B54" s="75" t="s">
-        <v>139</v>
+      <c r="B54" s="73" t="s">
+        <v>137</v>
       </c>
       <c r="C54" s="27" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A55" s="27"/>
-      <c r="B55" s="74" t="s">
+      <c r="B55" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="C55" s="29" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B56" s="74" t="s">
         <v>141</v>
       </c>
-      <c r="C55" s="29" t="s">
+      <c r="C56" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B56" s="76" t="s">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B57" s="74" t="s">
         <v>143</v>
       </c>
-      <c r="C56" t="s">
+      <c r="C57" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B57" s="76" t="s">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B58" s="74" t="s">
         <v>145</v>
       </c>
-      <c r="C57" t="s">
+      <c r="C58" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B58" s="76" t="s">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B59" s="74" t="s">
         <v>147</v>
       </c>
-      <c r="C58" t="s">
+      <c r="C59" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B59" s="76" t="s">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B60" s="74" t="s">
         <v>149</v>
       </c>
-      <c r="C59" t="s">
+      <c r="C60" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B60" s="76" t="s">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B61" s="74" t="s">
         <v>151</v>
       </c>
-      <c r="C60" t="s">
+      <c r="C61" t="s">
         <v>152</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B61" s="76" t="s">
-        <v>153</v>
-      </c>
-      <c r="C61" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="B62" s="172" t="s">
-        <v>56</v>
-      </c>
-      <c r="C62" s="173"/>
+        <v>46</v>
+      </c>
+      <c r="B62" s="118" t="s">
+        <v>54</v>
+      </c>
+      <c r="C62" s="119"/>
     </row>
     <row r="63" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A63" s="27"/>
-      <c r="B63" s="74" t="s">
-        <v>155</v>
+      <c r="B63" s="72" t="s">
+        <v>153</v>
       </c>
       <c r="C63" s="29" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A64" s="27"/>
-      <c r="B64" s="74" t="s">
-        <v>157</v>
+      <c r="B64" s="72" t="s">
+        <v>155</v>
       </c>
       <c r="C64" s="29" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A65" s="27"/>
-      <c r="B65" s="74" t="s">
+      <c r="B65" s="72" t="s">
+        <v>157</v>
+      </c>
+      <c r="C65" s="29" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B66" s="72" t="s">
         <v>159</v>
       </c>
-      <c r="C65" s="29" t="s">
+      <c r="C66" t="s">
         <v>160</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B66" s="74" t="s">
-        <v>161</v>
-      </c>
-      <c r="C66" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A67" s="26"/>
-      <c r="B67" s="75" t="s">
-        <v>163</v>
+      <c r="B67" s="73" t="s">
+        <v>161</v>
       </c>
       <c r="C67" s="27" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="68" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A68" s="27"/>
-      <c r="B68" s="74" t="s">
-        <v>165</v>
+      <c r="B68" s="72" t="s">
+        <v>163</v>
       </c>
       <c r="C68" s="29" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.2">
@@ -4220,8 +4117,8 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A71" s="26"/>
-      <c r="B71" s="172"/>
-      <c r="C71" s="173"/>
+      <c r="B71" s="118"/>
+      <c r="C71" s="119"/>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A72" s="27"/>
@@ -4240,8 +4137,8 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A76" s="26"/>
-      <c r="B76" s="172"/>
-      <c r="C76" s="173"/>
+      <c r="B76" s="118"/>
+      <c r="C76" s="119"/>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A77" s="27"/>
@@ -4266,6 +4163,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000B7BBE98651F7A43AC7BF2F06836443C" ma:contentTypeVersion="14" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="1e11716b46139950f2c3274e18a0400a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8103b6e4-b1cc-417b-af38-f980b3f4bdef" xmlns:ns3="026a8ae5-d6a9-4af7-bf98-fe61cc11d283" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0250f191272c0b89fb718059af881c7f" ns2:_="" ns3:_="">
     <xsd:import namespace="8103b6e4-b1cc-417b-af38-f980b3f4bdef"/>
@@ -4494,15 +4400,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -4515,6 +4412,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3B0F275-0B75-4410-A72C-AE1913414E16}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{85A46513-1514-4CC8-8F93-80F569849C66}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4533,14 +4438,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3B0F275-0B75-4410-A72C-AE1913414E16}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7F5217D-09D9-4B43-910D-375F05953276}">
   <ds:schemaRefs>

</xml_diff>